<commit_message>
Prepare company v2.0.1 source test updates
</commit_message>
<xml_diff>
--- a/config/A2700/Defaults_A2700M.xlsx
+++ b/config/A2700/Defaults_A2700M.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOYS\Documents\Claude\Projects\vision\VisionOCR\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PNT\61.AI\VisionOCR\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6E82E6-1BD3-403A-98C1-EB3D610E4F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3299FFBF-3355-441B-B1EA-E7154082AF46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-6216" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="setup_cases" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="227">
   <si>
     <t>name</t>
   </si>
@@ -226,9 +231,6 @@
     <t>51384, 1</t>
   </si>
   <si>
-    <t>15; 0</t>
-  </si>
-  <si>
     <t>Demand_NumSubInt</t>
   </si>
   <si>
@@ -698,6 +700,14 @@
   </si>
   <si>
     <t>120min</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>원래 기본값은 15</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1; 0</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1098,13 +1108,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H71"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.125" customWidth="1"/>
+    <col min="5" max="5" width="13.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1138,7 @@
       </c>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -1152,7 +1162,7 @@
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1175,7 +1185,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1198,7 +1208,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -1221,7 +1231,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1244,7 +1254,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1267,7 +1277,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1290,7 +1300,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1313,7 +1323,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1336,7 +1346,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1359,7 +1369,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -1382,7 +1392,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -1405,7 +1415,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -1428,7 +1438,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1451,7 +1461,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -1474,7 +1484,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -1497,7 +1507,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -1514,21 +1524,21 @@
         <v>17</v>
       </c>
       <c r="F18" t="s">
+        <v>226</v>
+      </c>
+      <c r="G18" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
         <v>68</v>
       </c>
-      <c r="G18">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="B19" t="b">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>69</v>
-      </c>
-      <c r="B19" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
-        <v>70</v>
       </c>
       <c r="D19" t="s">
         <v>16</v>
@@ -1543,15 +1553,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="b">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>71</v>
-      </c>
-      <c r="B20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
-        <v>72</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
@@ -1563,21 +1573,21 @@
         <v>44</v>
       </c>
       <c r="G20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="B21" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>74</v>
       </c>
-      <c r="B21" t="b">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>75</v>
-      </c>
-      <c r="D21" t="s">
-        <v>76</v>
       </c>
       <c r="E21" t="s">
         <v>17</v>
@@ -1586,67 +1596,67 @@
         <v>18</v>
       </c>
       <c r="G21" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="B22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>78</v>
       </c>
-      <c r="B22" t="b">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" t="s">
         <v>79</v>
       </c>
-      <c r="D22" t="s">
-        <v>76</v>
-      </c>
-      <c r="E22" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>80</v>
       </c>
-      <c r="G22" t="s">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="B23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>82</v>
       </c>
-      <c r="B23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" t="s">
         <v>83</v>
       </c>
-      <c r="D23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>84</v>
       </c>
-      <c r="G23" t="s">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="B24" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>86</v>
       </c>
-      <c r="B24" t="b">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
-        <v>87</v>
-      </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E24" t="s">
         <v>17</v>
@@ -1655,21 +1665,21 @@
         <v>18</v>
       </c>
       <c r="G24" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="B25" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>89</v>
       </c>
-      <c r="B25" t="b">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>90</v>
-      </c>
-      <c r="D25" t="s">
-        <v>91</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
@@ -1678,67 +1688,67 @@
         <v>18</v>
       </c>
       <c r="G25" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="B26" t="b">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>93</v>
       </c>
-      <c r="B26" t="b">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" t="s">
         <v>94</v>
       </c>
-      <c r="D26" t="s">
-        <v>91</v>
-      </c>
-      <c r="E26" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>95</v>
       </c>
-      <c r="G26" t="s">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="B27" t="b">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>97</v>
       </c>
-      <c r="B27" t="b">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
+        <v>90</v>
+      </c>
+      <c r="E27" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" t="s">
         <v>98</v>
       </c>
-      <c r="D27" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>99</v>
       </c>
-      <c r="G27" t="s">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="B28" t="b">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
         <v>101</v>
       </c>
-      <c r="B28" t="b">
-        <v>1</v>
-      </c>
-      <c r="C28" t="s">
-        <v>102</v>
-      </c>
       <c r="D28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E28" t="s">
         <v>17</v>
@@ -1747,205 +1757,205 @@
         <v>18</v>
       </c>
       <c r="G28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
         <v>103</v>
       </c>
-      <c r="B29" t="b">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" t="s">
         <v>104</v>
       </c>
-      <c r="D29" t="s">
-        <v>91</v>
-      </c>
-      <c r="E29" t="s">
-        <v>17</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>105</v>
       </c>
-      <c r="G29" t="s">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="B30" t="b">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
         <v>107</v>
       </c>
-      <c r="B30" t="b">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" t="s">
         <v>108</v>
       </c>
-      <c r="D30" t="s">
-        <v>91</v>
-      </c>
-      <c r="E30" t="s">
-        <v>17</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="G30" t="s">
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="B31" t="b">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
         <v>111</v>
       </c>
-      <c r="B31" t="b">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>112</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" t="s">
         <v>113</v>
       </c>
-      <c r="E31" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>114</v>
       </c>
-      <c r="G31" t="s">
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="B32" t="b">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
         <v>116</v>
       </c>
-      <c r="B32" t="b">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
+        <v>112</v>
+      </c>
+      <c r="E32" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" t="s">
+        <v>113</v>
+      </c>
+      <c r="G32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
         <v>117</v>
       </c>
-      <c r="D32" t="s">
+      <c r="B33" t="b">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>118</v>
+      </c>
+      <c r="D33" t="s">
+        <v>112</v>
+      </c>
+      <c r="E33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" t="s">
         <v>113</v>
       </c>
-      <c r="E32" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G33" t="s">
         <v>114</v>
       </c>
-      <c r="G32" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" t="b">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s">
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
         <v>119</v>
       </c>
-      <c r="D33" t="s">
+      <c r="B34" t="b">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34" t="s">
+        <v>112</v>
+      </c>
+      <c r="E34" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" t="s">
         <v>113</v>
       </c>
-      <c r="E33" t="s">
-        <v>17</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="G34" t="s">
         <v>114</v>
       </c>
-      <c r="G33" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>120</v>
-      </c>
-      <c r="B34" t="b">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
         <v>121</v>
       </c>
-      <c r="D34" t="s">
+      <c r="B35" t="b">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>122</v>
+      </c>
+      <c r="D35" t="s">
+        <v>123</v>
+      </c>
+      <c r="E35" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" t="s">
+        <v>124</v>
+      </c>
+      <c r="G35" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" t="b">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>127</v>
+      </c>
+      <c r="D36" t="s">
+        <v>123</v>
+      </c>
+      <c r="E36" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" t="s">
         <v>113</v>
       </c>
-      <c r="E34" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G36" t="s">
         <v>114</v>
       </c>
-      <c r="G34" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>122</v>
-      </c>
-      <c r="B35" t="b">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" t="b">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>129</v>
+      </c>
+      <c r="D37" t="s">
         <v>123</v>
-      </c>
-      <c r="D35" t="s">
-        <v>124</v>
-      </c>
-      <c r="E35" t="s">
-        <v>17</v>
-      </c>
-      <c r="F35" t="s">
-        <v>125</v>
-      </c>
-      <c r="G35" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>127</v>
-      </c>
-      <c r="B36" t="b">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>128</v>
-      </c>
-      <c r="D36" t="s">
-        <v>124</v>
-      </c>
-      <c r="E36" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" t="s">
-        <v>114</v>
-      </c>
-      <c r="G36" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>129</v>
-      </c>
-      <c r="B37" t="b">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s">
-        <v>130</v>
-      </c>
-      <c r="D37" t="s">
-        <v>124</v>
       </c>
       <c r="E37" t="s">
         <v>17</v>
@@ -1954,228 +1964,228 @@
         <v>31</v>
       </c>
       <c r="G37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="B38" t="b">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
         <v>132</v>
       </c>
-      <c r="B38" t="b">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
+        <v>123</v>
+      </c>
+      <c r="E38" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" t="s">
         <v>133</v>
       </c>
-      <c r="D38" t="s">
-        <v>124</v>
-      </c>
-      <c r="E38" t="s">
-        <v>17</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>134</v>
       </c>
-      <c r="G38" t="s">
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="B39" t="b">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
         <v>136</v>
       </c>
-      <c r="B39" t="b">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" t="s">
+        <v>113</v>
+      </c>
+      <c r="G39" t="s">
         <v>137</v>
       </c>
-      <c r="D39" t="s">
-        <v>124</v>
-      </c>
-      <c r="E39" t="s">
-        <v>17</v>
-      </c>
-      <c r="F39" t="s">
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" t="b">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" t="s">
+        <v>123</v>
+      </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" t="s">
         <v>114</v>
       </c>
-      <c r="G39" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>139</v>
-      </c>
-      <c r="B40" t="b">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
         <v>140</v>
       </c>
-      <c r="D40" t="s">
-        <v>124</v>
-      </c>
-      <c r="E40" t="s">
-        <v>17</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="B41" t="b">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>141</v>
+      </c>
+      <c r="D41" t="s">
+        <v>123</v>
+      </c>
+      <c r="E41" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" t="s">
+        <v>113</v>
+      </c>
+      <c r="G41" t="s">
         <v>114</v>
       </c>
-      <c r="G40" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>141</v>
-      </c>
-      <c r="B41" t="b">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s">
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
         <v>142</v>
       </c>
-      <c r="D41" t="s">
-        <v>124</v>
-      </c>
-      <c r="E41" t="s">
-        <v>17</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="B42" t="b">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>143</v>
+      </c>
+      <c r="D42" t="s">
+        <v>123</v>
+      </c>
+      <c r="E42" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" t="s">
+        <v>113</v>
+      </c>
+      <c r="G42" t="s">
         <v>114</v>
       </c>
-      <c r="G41" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>143</v>
-      </c>
-      <c r="B42" t="b">
-        <v>1</v>
-      </c>
-      <c r="C42" t="s">
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
         <v>144</v>
       </c>
-      <c r="D42" t="s">
-        <v>124</v>
-      </c>
-      <c r="E42" t="s">
-        <v>17</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="B43" t="b">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>145</v>
+      </c>
+      <c r="D43" t="s">
+        <v>123</v>
+      </c>
+      <c r="E43" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" t="s">
+        <v>113</v>
+      </c>
+      <c r="G43" t="s">
         <v>114</v>
       </c>
-      <c r="G42" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>145</v>
-      </c>
-      <c r="B43" t="b">
-        <v>1</v>
-      </c>
-      <c r="C43" t="s">
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
         <v>146</v>
       </c>
-      <c r="D43" t="s">
-        <v>124</v>
-      </c>
-      <c r="E43" t="s">
-        <v>17</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="B44" t="b">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>147</v>
+      </c>
+      <c r="D44" t="s">
+        <v>123</v>
+      </c>
+      <c r="E44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" t="s">
+        <v>113</v>
+      </c>
+      <c r="G44" t="s">
         <v>114</v>
       </c>
-      <c r="G43" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>147</v>
-      </c>
-      <c r="B44" t="b">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
         <v>148</v>
       </c>
-      <c r="D44" t="s">
-        <v>124</v>
-      </c>
-      <c r="E44" t="s">
-        <v>17</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="B45" t="b">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D45" t="s">
+        <v>123</v>
+      </c>
+      <c r="E45" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" t="s">
+        <v>113</v>
+      </c>
+      <c r="G45" t="s">
         <v>114</v>
       </c>
-      <c r="G44" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>149</v>
-      </c>
-      <c r="B45" t="b">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
         <v>150</v>
       </c>
-      <c r="D45" t="s">
-        <v>124</v>
-      </c>
-      <c r="E45" t="s">
-        <v>17</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="B46" t="b">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" t="s">
+        <v>123</v>
+      </c>
+      <c r="E46" t="s">
+        <v>17</v>
+      </c>
+      <c r="F46" t="s">
+        <v>113</v>
+      </c>
+      <c r="G46" t="s">
         <v>114</v>
       </c>
-      <c r="G45" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>151</v>
-      </c>
-      <c r="B46" t="b">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s">
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
         <v>152</v>
       </c>
-      <c r="D46" t="s">
-        <v>124</v>
-      </c>
-      <c r="E46" t="s">
-        <v>17</v>
-      </c>
-      <c r="F46" t="s">
-        <v>114</v>
-      </c>
-      <c r="G46" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+      <c r="B47" t="b">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
         <v>153</v>
       </c>
-      <c r="B47" t="b">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>154</v>
-      </c>
       <c r="D47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E47" t="s">
         <v>17</v>
@@ -2184,44 +2194,44 @@
         <v>31</v>
       </c>
       <c r="G47" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
+        <v>154</v>
+      </c>
+      <c r="B48" t="b">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
         <v>155</v>
       </c>
-      <c r="B48" t="b">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
+        <v>123</v>
+      </c>
+      <c r="E48" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" t="s">
+        <v>113</v>
+      </c>
+      <c r="G48" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
         <v>156</v>
       </c>
-      <c r="D48" t="s">
-        <v>124</v>
-      </c>
-      <c r="E48" t="s">
-        <v>17</v>
-      </c>
-      <c r="F48" t="s">
-        <v>114</v>
-      </c>
-      <c r="G48" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+      <c r="B49" t="b">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
         <v>157</v>
       </c>
-      <c r="B49" t="b">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s">
-        <v>158</v>
-      </c>
       <c r="D49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E49" t="s">
         <v>17</v>
@@ -2230,44 +2240,44 @@
         <v>31</v>
       </c>
       <c r="G49" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
+        <v>158</v>
+      </c>
+      <c r="B50" t="b">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
         <v>159</v>
       </c>
-      <c r="B50" t="b">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
+        <v>123</v>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+      <c r="F50" t="s">
+        <v>113</v>
+      </c>
+      <c r="G50" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
         <v>160</v>
       </c>
-      <c r="D50" t="s">
-        <v>124</v>
-      </c>
-      <c r="E50" t="s">
-        <v>17</v>
-      </c>
-      <c r="F50" t="s">
-        <v>114</v>
-      </c>
-      <c r="G50" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="B51" t="b">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
         <v>161</v>
       </c>
-      <c r="B51" t="b">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>162</v>
-      </c>
       <c r="D51" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E51" t="s">
         <v>17</v>
@@ -2276,21 +2286,21 @@
         <v>31</v>
       </c>
       <c r="G51" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
+        <v>162</v>
+      </c>
+      <c r="B52" t="b">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
         <v>163</v>
       </c>
-      <c r="B52" t="b">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>164</v>
-      </c>
-      <c r="D52" t="s">
-        <v>165</v>
       </c>
       <c r="E52" t="s">
         <v>17</v>
@@ -2299,21 +2309,21 @@
         <v>18</v>
       </c>
       <c r="G52" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="B53" t="b">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
         <v>167</v>
       </c>
-      <c r="B53" t="b">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s">
-        <v>168</v>
-      </c>
       <c r="D53" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E53" t="s">
         <v>17</v>
@@ -2322,44 +2332,44 @@
         <v>18</v>
       </c>
       <c r="G53" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
+      <c r="B54" t="b">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
         <v>170</v>
       </c>
-      <c r="B54" t="b">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>171</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>172</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>173</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>174</v>
       </c>
-      <c r="G54" t="s">
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+      <c r="B55" t="b">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
         <v>176</v>
       </c>
-      <c r="B55" t="b">
-        <v>1</v>
-      </c>
-      <c r="C55" t="s">
-        <v>177</v>
-      </c>
       <c r="D55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E55" t="s">
         <v>17</v>
@@ -2368,67 +2378,67 @@
         <v>18</v>
       </c>
       <c r="G55" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
+        <v>177</v>
+      </c>
+      <c r="B56" t="b">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
         <v>178</v>
       </c>
-      <c r="B56" t="b">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
+        <v>171</v>
+      </c>
+      <c r="E56" t="s">
+        <v>17</v>
+      </c>
+      <c r="F56" t="s">
+        <v>79</v>
+      </c>
+      <c r="G56" t="s">
         <v>179</v>
       </c>
-      <c r="D56" t="s">
-        <v>172</v>
-      </c>
-      <c r="E56" t="s">
-        <v>17</v>
-      </c>
-      <c r="F56" t="s">
-        <v>80</v>
-      </c>
-      <c r="G56" t="s">
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
+      <c r="B57" t="b">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
         <v>181</v>
       </c>
-      <c r="B57" t="b">
-        <v>1</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
+        <v>171</v>
+      </c>
+      <c r="E57" t="s">
+        <v>17</v>
+      </c>
+      <c r="F57" t="s">
+        <v>83</v>
+      </c>
+      <c r="G57" t="s">
         <v>182</v>
       </c>
-      <c r="D57" t="s">
-        <v>172</v>
-      </c>
-      <c r="E57" t="s">
-        <v>17</v>
-      </c>
-      <c r="F57" t="s">
-        <v>84</v>
-      </c>
-      <c r="G57" t="s">
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+      <c r="B58" t="b">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
         <v>184</v>
       </c>
-      <c r="B58" t="b">
-        <v>1</v>
-      </c>
-      <c r="C58" t="s">
-        <v>185</v>
-      </c>
       <c r="D58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E58" t="s">
         <v>17</v>
@@ -2437,90 +2447,90 @@
         <v>18</v>
       </c>
       <c r="G58" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A59" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+      <c r="B59" t="b">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
         <v>187</v>
       </c>
-      <c r="B59" t="b">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
+        <v>171</v>
+      </c>
+      <c r="E59" t="s">
+        <v>17</v>
+      </c>
+      <c r="F59" t="s">
         <v>188</v>
       </c>
-      <c r="D59" t="s">
-        <v>172</v>
-      </c>
-      <c r="E59" t="s">
-        <v>17</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="G59" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
+      <c r="B60" t="b">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
         <v>190</v>
       </c>
-      <c r="B60" t="b">
-        <v>1</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
+        <v>171</v>
+      </c>
+      <c r="E60" t="s">
+        <v>17</v>
+      </c>
+      <c r="F60" t="s">
         <v>191</v>
       </c>
-      <c r="D60" t="s">
-        <v>172</v>
-      </c>
-      <c r="E60" t="s">
-        <v>17</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
         <v>192</v>
       </c>
-      <c r="G60" t="s">
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A61" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
+      <c r="B61" t="b">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
         <v>194</v>
       </c>
-      <c r="B61" t="b">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
+        <v>171</v>
+      </c>
+      <c r="E61" t="s">
+        <v>17</v>
+      </c>
+      <c r="F61" t="s">
+        <v>124</v>
+      </c>
+      <c r="G61" t="s">
         <v>195</v>
       </c>
-      <c r="D61" t="s">
-        <v>172</v>
-      </c>
-      <c r="E61" t="s">
-        <v>17</v>
-      </c>
-      <c r="F61" t="s">
-        <v>125</v>
-      </c>
-      <c r="G61" t="s">
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A62" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+      <c r="B62" t="b">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
         <v>197</v>
       </c>
-      <c r="B62" t="b">
-        <v>1</v>
-      </c>
-      <c r="C62" t="s">
-        <v>198</v>
-      </c>
       <c r="D62" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E62" t="s">
         <v>17</v>
@@ -2529,90 +2539,90 @@
         <v>18</v>
       </c>
       <c r="G62" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
+        <v>198</v>
+      </c>
+      <c r="B63" t="b">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
         <v>199</v>
       </c>
-      <c r="B63" t="b">
-        <v>1</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
+        <v>171</v>
+      </c>
+      <c r="E63" t="s">
+        <v>17</v>
+      </c>
+      <c r="F63" t="s">
+        <v>188</v>
+      </c>
+      <c r="G63" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A64" t="s">
         <v>200</v>
       </c>
-      <c r="D63" t="s">
-        <v>172</v>
-      </c>
-      <c r="E63" t="s">
-        <v>17</v>
-      </c>
-      <c r="F63" t="s">
-        <v>189</v>
-      </c>
-      <c r="G63" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+      <c r="B64" t="b">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
         <v>201</v>
       </c>
-      <c r="B64" t="b">
-        <v>1</v>
-      </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
+        <v>171</v>
+      </c>
+      <c r="E64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F64" t="s">
         <v>202</v>
       </c>
-      <c r="D64" t="s">
-        <v>172</v>
-      </c>
-      <c r="E64" t="s">
-        <v>17</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
         <v>203</v>
       </c>
-      <c r="G64" t="s">
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A65" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
+      <c r="B65" t="b">
+        <v>1</v>
+      </c>
+      <c r="C65" t="s">
         <v>205</v>
       </c>
-      <c r="B65" t="b">
-        <v>1</v>
-      </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>206</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
+        <v>17</v>
+      </c>
+      <c r="F65" t="s">
+        <v>124</v>
+      </c>
+      <c r="G65" t="s">
         <v>207</v>
       </c>
-      <c r="E65" t="s">
-        <v>17</v>
-      </c>
-      <c r="F65" t="s">
-        <v>125</v>
-      </c>
-      <c r="G65" t="s">
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A66" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
+      <c r="B66" t="b">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
         <v>209</v>
       </c>
-      <c r="B66" t="b">
-        <v>1</v>
-      </c>
-      <c r="C66" t="s">
-        <v>210</v>
-      </c>
       <c r="D66" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E66" t="s">
         <v>17</v>
@@ -2621,122 +2631,122 @@
         <v>18</v>
       </c>
       <c r="G66" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A67" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
+      <c r="B67" t="b">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
         <v>212</v>
       </c>
-      <c r="B67" t="b">
-        <v>1</v>
-      </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>213</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>214</v>
-      </c>
-      <c r="E67" t="s">
-        <v>215</v>
       </c>
       <c r="F67" t="s">
         <v>18</v>
       </c>
       <c r="G67" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A68" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
+      <c r="B68" t="b">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
         <v>217</v>
       </c>
-      <c r="B68" t="b">
-        <v>1</v>
-      </c>
-      <c r="C68" t="s">
-        <v>218</v>
-      </c>
       <c r="D68" t="s">
+        <v>213</v>
+      </c>
+      <c r="E68" t="s">
         <v>214</v>
-      </c>
-      <c r="E68" t="s">
-        <v>215</v>
       </c>
       <c r="F68" t="s">
         <v>18</v>
       </c>
       <c r="G68" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
+        <v>218</v>
+      </c>
+      <c r="B69" t="b">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
         <v>219</v>
       </c>
-      <c r="B69" t="b">
-        <v>1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>220</v>
-      </c>
       <c r="D69" t="s">
+        <v>213</v>
+      </c>
+      <c r="E69" t="s">
         <v>214</v>
-      </c>
-      <c r="E69" t="s">
-        <v>215</v>
       </c>
       <c r="F69" t="s">
         <v>18</v>
       </c>
       <c r="G69" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
+        <v>220</v>
+      </c>
+      <c r="B70" t="b">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
         <v>221</v>
       </c>
-      <c r="B70" t="b">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s">
-        <v>222</v>
-      </c>
       <c r="D70" t="s">
+        <v>213</v>
+      </c>
+      <c r="E70" t="s">
         <v>214</v>
-      </c>
-      <c r="E70" t="s">
-        <v>215</v>
       </c>
       <c r="F70" t="s">
         <v>18</v>
       </c>
       <c r="G70" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
+        <v>222</v>
+      </c>
+      <c r="B71" t="b">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
         <v>223</v>
       </c>
-      <c r="B71" t="b">
-        <v>1</v>
-      </c>
-      <c r="C71" t="s">
-        <v>224</v>
-      </c>
       <c r="D71" t="s">
+        <v>213</v>
+      </c>
+      <c r="E71" t="s">
         <v>214</v>
-      </c>
-      <c r="E71" t="s">
-        <v>215</v>
       </c>
       <c r="F71" t="s">
         <v>18</v>
       </c>
       <c r="G71" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>